<commit_message>
Étape 1C : liste des médicaments et ordonnance A5/A4 (Médic.), enregistrée dans la consultation du jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/listes/Medicaments_Onco360.xlsx
+++ b/listes/Medicaments_Onco360.xlsx
@@ -5,7 +5,7 @@
     <sheet name="Médicaments" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Médicaments!$A$1:$C$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Médicaments!$A$1:$C$166</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -24,7 +24,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -34,11 +34,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF3563B0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDFF3E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,15 +57,12 @@
   <cellStyleXfs count="1">
     <xf/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf/>
     <xf fontId="1" fillId="2" borderId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -171,17 +163,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr" s="3">
+      <c r="A6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">ANDROCUR (cyprotérone) 50 mg</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="3">
+      <c r="B6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">2 comprimés matin et soir (soit 4 comprimés = 200 mg par jour), à commencer 1 semaine avant la 1re injection d'agoniste de la LH-RH, pendant 3 semaines au total</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="3">
+      <c r="C6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Hormonothérapie anticancéreuse (anti-androgène)</t>
         </is>
@@ -222,34 +214,34 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr" s="3">
+      <c r="A9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">ARIMIDEX (anastrozole) 1 mg</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="3">
+      <c r="B9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 comprimé par jour, à heure fixe, pendant 3 mois</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="3">
+      <c r="C9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Hormonothérapie anticancéreuse (anti-aromatase)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr" s="3">
+      <c r="A10" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">AROMASINE (exémestane) 25 mg</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr" s="3">
+      <c r="B10" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 comprimé par jour, après un repas, à heure fixe, pendant 3 mois</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr" s="3">
+      <c r="C10" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Hormonothérapie anticancéreuse (anti-aromatase)</t>
         </is>
@@ -324,17 +316,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr" s="3">
+      <c r="A15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">BIAFINE émulsion (trolamine)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr" s="3">
+      <c r="B15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">2 à 3 applications par jour en couche épaisse sur la zone irradiée, à faire pénétrer par un léger massage ; pas d'application dans les 2 heures qui précèdent la séance</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr" s="3">
+      <c r="C15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Soin de la radiodermite</t>
         </is>
@@ -409,34 +401,34 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr" s="3">
+      <c r="A20" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">CAPÉCITABINE (XELODA) 500 mg / 150 mg</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr" s="3">
+      <c r="B20" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">… comprimés de 500 mg et … comprimés de 150 mg le matin et le soir (… mg/m² 2 fois par jour), dans les 30 minutes qui suivent le repas, de J1 à J14, puis 7 jours d'arrêt (reprise à J22)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr" s="3">
+      <c r="C20" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Chimiothérapie orale (fluoropyrimidine)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr" s="3">
+      <c r="A21" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">CAPÉCITABINE (XELODA) 500 mg / 150 mg, avec la radiothérapie</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr" s="3">
+      <c r="B21" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">… comprimés de 500 mg et … comprimés de 150 mg le matin et le soir (825 mg/m² 2 fois par jour), dans les 30 minutes qui suivent le repas, chaque jour de radiothérapie</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr" s="3">
+      <c r="C21" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Chimiothérapie orale (fluoropyrimidine)</t>
         </is>
@@ -654,7 +646,7 @@
       </c>
       <c r="B34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 injection tous les 3 mois</t>
+          <t xml:space="preserve">1 injection intramusculaire tous les 3 mois</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="2">
@@ -671,7 +663,7 @@
       </c>
       <c r="B35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 injection tous les 6 mois</t>
+          <t xml:space="preserve">1 injection intramusculaire tous les 6 mois</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="2">
@@ -681,51 +673,51 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr" s="3">
+      <c r="A36" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">DECAPEPTYL LP (triptoréline) 3 mg</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr" s="3">
+      <c r="B36" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 injection intramusculaire tous les 28 jours</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr" s="3">
+      <c r="C36" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Hormonothérapie anticancéreuse (agoniste de la LH-RH)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr" s="3">
+      <c r="A37" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">DEXAMÉTHASONE 4 mg, comprimé</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr" s="3">
+      <c r="B37" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">2 comprimés le matin (soit 8 mg) à J2 et J3 après la chimiothérapie</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr" s="3">
+      <c r="C37" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Corticoïde (antiémétique)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr" s="3">
+      <c r="A38" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">DEXAMÉTHASONE 4 mg, comprimé (œdème cérébral)</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr" s="3">
+      <c r="B38" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">… comprimés le matin (… mg par jour), puis diminution progressive selon l'évolution</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr" s="3">
+      <c r="C38" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Corticoïde</t>
         </is>
@@ -834,17 +826,17 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr" s="3">
+      <c r="A45" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">DUROGESIC (fentanyl) 12 / 25 / 50 µg/h, patch</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr" s="3">
+      <c r="B45" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 patch à changer toutes les 72 heures (3 jours)</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr" s="3">
+      <c r="C45" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Antalgique de palier 3 (opioïde transdermique)</t>
         </is>
@@ -902,17 +894,17 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr" s="3">
+      <c r="A49" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">ENDOXAN (cyclophosphamide) 50 mg</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr" s="3">
+      <c r="B49" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 comprimé par jour, le matin, avec un grand verre d'eau (chimiothérapie métronomique)</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr" s="3">
+      <c r="C49" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Chimiothérapie orale (agent alkylant)</t>
         </is>
@@ -987,17 +979,17 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr" s="3">
+      <c r="A54" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">FASLODEX (fulvestrant) 250 mg</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr" s="3">
+      <c r="B54" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">2 injections intramusculaires lentes (1 dans chaque fesse, soit 500 mg) à J1, J15 et J29, puis tous les mois</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr" s="3">
+      <c r="C54" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Hormonothérapie anticancéreuse (anti-œstrogène)</t>
         </is>
@@ -1242,17 +1234,17 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr" s="3">
+      <c r="A69" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">GLIVEC (imatinib) 400 mg</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr" s="3">
+      <c r="B69" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 comprimé par jour, au cours d'un repas, avec un grand verre d'eau</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr" s="3">
+      <c r="C69" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Thérapie ciblée (inhibiteur de tyrosine kinase)</t>
         </is>
@@ -1361,439 +1353,439 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr" s="3">
+      <c r="A76" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">IBRANCE (palbociclib) 125 mg</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr" s="3">
+      <c r="B76" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 par jour, à heure fixe, au cours d'un repas, pendant 21 jours, puis 7 jours d'arrêt (cycle de 28 jours), avec l'hormonothérapie</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr" s="3">
+      <c r="C76" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Thérapie ciblée (inhibiteur de CDK4/6)</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr" s="3">
+      <c r="A77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">IMFINZI (durvalumab) 500 mg</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3 flacons de 500 mg (1 500 mg) tous les 28 jours, pendant 12 mois au maximum</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Immunothérapie</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">KEPPRA (lévétiracétam) 500 mg</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr" s="3">
+      <c r="B78" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 comprimé matin et soir (soit 2 comprimés par jour)</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr" s="3">
+      <c r="C78" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Antiépileptique</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">KISQALI (ribociclib) 200 mg</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">3 comprimés (600 mg) en une prise par jour, à heure fixe, pendant 21 jours, puis 7 jours d'arrêt (cycle de 28 jours), avec l'hormonothérapie</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Thérapie ciblée (inhibiteur de CDK4/6)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">KIT DE DILATATEURS VAGINAUX (4 tailles)</t>
+          <t xml:space="preserve">KEYTRUDA (pembrolizumab) 100 mg</t>
         </is>
       </c>
       <c r="B79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Dilatation vaginale progressive (commencer par le plus petit), 2 à 3 fois par semaine, 10 minutes par séance</t>
+          <t xml:space="preserve">2 flacons de 100 mg tous les 21 jours</t>
         </is>
       </c>
       <c r="C79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Dispositif médical</t>
+          <t xml:space="preserve">Immunothérapie</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">KLEAN PREP</t>
+          <t xml:space="preserve">KISQALI (ribociclib) 200 mg</t>
         </is>
       </c>
       <c r="B80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">4 sachets dans 4 litres d'eau : 2 litres entre 18 h et 20 h la veille, puis 2 litres entre 0 h et 2 h le jour de l'examen</t>
+          <t xml:space="preserve">3 comprimés (600 mg) en une prise par jour, à heure fixe, pendant 21 jours, puis 7 jours d'arrêt (cycle de 28 jours), avec l'hormonothérapie</t>
         </is>
       </c>
       <c r="C80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Préparation colique (laxatif osmotique)</t>
+          <t xml:space="preserve">Thérapie ciblée (inhibiteur de CDK4/6)</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">LEVOTHYROX (lévothyroxine) 25 / 50 / 100 µg</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 comprimé le matin à jeun, 30 minutes avant le petit-déjeuner</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Hormone thyroïdienne</t>
+      <c r="A81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">KIT DE DILATATEURS VAGINAUX (4 tailles)</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Dilatation vaginale progressive (commencer par le plus petit), 2 à 3 fois par semaine, 10 minutes par séance</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Dispositif médical</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LIXIFOR, gélule</t>
+          <t xml:space="preserve">KLEAN PREP</t>
         </is>
       </c>
       <c r="B82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 gélule le soir au coucher avec un grand verre d'eau</t>
+          <t xml:space="preserve">4 sachets dans 4 litres d'eau : 2 litres entre 18 h et 20 h la veille, puis 2 litres entre 0 h et 2 h le jour de l'examen</t>
         </is>
       </c>
       <c r="C82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Complément alimentaire (transit intestinal, plantes)</t>
+          <t xml:space="preserve">Préparation colique (laxatif osmotique)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LOMEXINE (fenticonazole) 2 % crème vulvaire</t>
+          <t xml:space="preserve">LEVOTHYROX (lévothyroxine) 25 / 50 / 100 µg</t>
         </is>
       </c>
       <c r="B83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 application matin et soir (soit 2 par jour) pendant 1 semaine</t>
+          <t xml:space="preserve">1 comprimé le matin à jeun, 30 minutes avant le petit-déjeuner</t>
         </is>
       </c>
       <c r="C83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antifongique local</t>
+          <t xml:space="preserve">Hormone thyroïdienne</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LOMEXINE (fenticonazole) 600 mg ovule</t>
+          <t xml:space="preserve">LIXIFOR, gélule</t>
         </is>
       </c>
       <c r="B84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 ovule le soir au coucher, en une seule fois (dose unique)</t>
+          <t xml:space="preserve">1 gélule le soir au coucher avec un grand verre d'eau</t>
         </is>
       </c>
       <c r="C84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antifongique gynécologique</t>
+          <t xml:space="preserve">Complément alimentaire (transit intestinal, plantes)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">LOMEXINE (fenticonazole) 2 % crème vulvaire</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 application matin et soir (soit 2 par jour) pendant 1 semaine</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Antifongique local</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LOMEXINE (fenticonazole) 600 mg ovule</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 ovule le soir au coucher, en une seule fois (dose unique)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Antifongique gynécologique</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">LOPERIUM (lopéramide) 2 mg</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr" s="2">
+      <c r="B87" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 à 2 comprimés en cas de diarrhée importante, maximum 6 comprimés par jour</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr" s="2">
+      <c r="C87" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Antidiarrhéique</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">LOVENOX (énoxaparine) 4 000 UI / 0,4 ml</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 injection sous-cutanée par jour pendant … jours</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Anticoagulant (héparine de bas poids moléculaire), prévention</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">LYNPARZA (olaparib) 150 mg</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">2 comprimés matin et soir (soit 4 comprimés = 600 mg par jour), en continu</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Thérapie ciblée (inhibiteur de PARP)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LYRICA (prégabaline) 50 mg</t>
+          <t xml:space="preserve">LOVENOX (énoxaparine) 4 000 UI / 0,4 ml</t>
         </is>
       </c>
       <c r="B88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé matin et soir (soit 2 comprimés = 100 mg par jour) pour commencer</t>
+          <t xml:space="preserve">1 injection sous-cutanée par jour pendant … jours</t>
         </is>
       </c>
       <c r="C88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antiépileptique (douleurs neuropathiques)</t>
+          <t xml:space="preserve">Anticoagulant (héparine de bas poids moléculaire), prévention</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MAGMINE (magnésium + vitamine B6)</t>
+          <t xml:space="preserve">LYNPARZA (olaparib) 150 mg</t>
         </is>
       </c>
       <c r="B89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé le matin</t>
+          <t xml:space="preserve">2 comprimés matin et soir (soit 4 comprimés = 600 mg par jour), en continu</t>
         </is>
       </c>
       <c r="C89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Supplément en magnésium</t>
+          <t xml:space="preserve">Thérapie ciblée (inhibiteur de PARP)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MEPILEX EM / TRANSFER (pansement hydrocellulaire)</t>
+          <t xml:space="preserve">LYRICA (prégabaline) 50 mg</t>
         </is>
       </c>
       <c r="B90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 pansement, à changer tous les jours après nettoyage soigneux</t>
+          <t xml:space="preserve">1 comprimé matin et soir (soit 2 comprimés = 100 mg par jour) pour commencer</t>
         </is>
       </c>
       <c r="C90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Dispositif médical (pansement)</t>
+          <t xml:space="preserve">Antiépileptique (douleurs neuropathiques)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MORIDIL pommade</t>
+          <t xml:space="preserve">MAGMINE (magnésium + vitamine B6)</t>
         </is>
       </c>
       <c r="B91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 application 2 fois par jour (matin et soir) sur la zone anale</t>
+          <t xml:space="preserve">1 comprimé le matin</t>
         </is>
       </c>
       <c r="C91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antihémorroïdaire (lidocaïne)</t>
+          <t xml:space="preserve">Supplément en magnésium</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MORIDIL suppositoire</t>
+          <t xml:space="preserve">MEPILEX EM / TRANSFER (pansement hydrocellulaire)</t>
         </is>
       </c>
       <c r="B92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 suppositoire enduit de pommade, 2 fois par jour</t>
+          <t xml:space="preserve">1 pansement, à changer tous les jours après nettoyage soigneux</t>
         </is>
       </c>
       <c r="C92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antihémorroïdaire (lidocaïne)</t>
+          <t xml:space="preserve">Dispositif médical (pansement)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MOSCONTIN LP (sulfate de morphine) 10 / 30 / 60 / 100 mg</t>
+          <t xml:space="preserve">MORIDIL pommade</t>
         </is>
       </c>
       <c r="B93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé le matin et 1 le soir (toutes les 12 heures)</t>
+          <t xml:space="preserve">1 application 2 fois par jour (matin et soir) sur la zone anale</t>
         </is>
       </c>
       <c r="C93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antalgique de palier 3 (morphine à libération prolongée)</t>
+          <t xml:space="preserve">Antihémorroïdaire (lidocaïne)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MOTILIUM (dompéridone) sirop</t>
+          <t xml:space="preserve">MORIDIL suppositoire</t>
         </is>
       </c>
       <c r="B94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 cuillère-mesure 3 fois par jour, 15 minutes avant les repas, pendant 3 jours</t>
+          <t xml:space="preserve">1 suppositoire enduit de pommade, 2 fois par jour</t>
         </is>
       </c>
       <c r="C94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antiémétique (antidopaminergique)</t>
+          <t xml:space="preserve">Antihémorroïdaire (lidocaïne)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MOVICOL (macrogol)</t>
+          <t xml:space="preserve">MOSCONTIN LP (sulfate de morphine) 10 / 30 / 60 / 100 mg</t>
         </is>
       </c>
       <c r="B95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 sachet matin et soir (soit 2 sachets par jour) en cas de constipation importante</t>
+          <t xml:space="preserve">1 comprimé le matin et 1 le soir (toutes les 12 heures)</t>
         </is>
       </c>
       <c r="C95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Laxatif osmotique</t>
+          <t xml:space="preserve">Antalgique de palier 3 (morphine à libération prolongée)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">MOTILIUM (dompéridone) sirop</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 cuillère-mesure 3 fois par jour, 15 minutes avant les repas, pendant 3 jours</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Antiémétique (antidopaminergique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MOVICOL (macrogol)</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 sachet matin et soir (soit 2 sachets par jour) en cas de constipation importante</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Laxatif osmotique</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">MYCODERME pommade</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr" s="2">
+      <c r="B98" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">1 application 2 fois par jour (matin et soir) pendant 3 semaines</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr" s="2">
+      <c r="C98" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Antifongique local</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">NAVELBINE (vinorelbine) 20 mg / 30 mg, capsule molle</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">… capsules de 20 mg et … capsules de 30 mg en une prise, 1 fois par semaine (60 à 80 mg/m²), au cours d'un repas léger, avalées entières avec un verre d'eau, sans les mâcher</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Chimiothérapie orale (vinca-alcaloïde)</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">NEULASTIM (pegfilgrastim) 6 mg</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 injection sous-cutanée par cycle, 24 heures après la fin de la chimiothérapie (J2)</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Facteur de croissance (G-CSF à action prolongée)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">NEUPOGEN (filgrastim) 48 MU</t>
+          <t xml:space="preserve">NAVELBINE (vinorelbine) 20 mg / 30 mg, capsule molle</t>
         </is>
       </c>
       <c r="B99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 injection sous-cutanée par jour pendant 5 jours (de J2 à J6 après la chimiothérapie)</t>
+          <t xml:space="preserve">… capsules de 20 mg et … capsules de 30 mg en une prise, 1 fois par semaine (60 à 80 mg/m²), au cours d'un repas léger, avalées entières avec un verre d'eau, sans les mâcher</t>
         </is>
       </c>
       <c r="C99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Facteur de croissance (G-CSF)</t>
+          <t xml:space="preserve">Chimiothérapie orale (vinca-alcaloïde)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">NIBIOL FORTE (nitroxoline) 100 mg</t>
+          <t xml:space="preserve">NEULASTIM (pegfilgrastim) 6 mg</t>
         </is>
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé matin, midi et soir (soit 3 comprimés par jour) pendant 10 jours</t>
+          <t xml:space="preserve">1 injection sous-cutanée par cycle, 24 heures après la fin de la chimiothérapie (J2)</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antiseptique urinaire</t>
+          <t xml:space="preserve">Facteur de croissance (G-CSF à action prolongée)</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">NIVESTIM (filgrastim) 30 MU</t>
+          <t xml:space="preserve">NEUPOGEN (filgrastim) 48 MU</t>
         </is>
       </c>
       <c r="B101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 injection sous-cutanée par jour pendant 3 jours (de J2 à J4 après la chimiothérapie)</t>
+          <t xml:space="preserve">1 injection sous-cutanée par jour pendant 5 jours (de J2 à J6 après la chimiothérapie)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr" s="2">
@@ -1805,1058 +1797,1109 @@
     <row r="102">
       <c r="A102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">NOCAND 50 mg</t>
+          <t xml:space="preserve">NIBIOL FORTE (nitroxoline) 100 mg</t>
         </is>
       </c>
       <c r="B102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé le matin pendant 7 jours</t>
+          <t xml:space="preserve">1 comprimé matin, midi et soir (soit 3 comprimés par jour) pendant 10 jours</t>
         </is>
       </c>
       <c r="C102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Antiseptique urinaire</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">NORMACOL lavement</t>
+          <t xml:space="preserve">NIVESTIM (filgrastim) 30 MU</t>
         </is>
       </c>
       <c r="B103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 lavement en l'absence de selles pendant 3 jours malgré les autres traitements (MOVICOL…)</t>
+          <t xml:space="preserve">1 injection sous-cutanée par jour pendant 3 jours (de J2 à J4 après la chimiothérapie)</t>
         </is>
       </c>
       <c r="C103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Laxatif (lavement rectal)</t>
+          <t xml:space="preserve">Facteur de croissance (G-CSF)</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OEDES (oméprazole) 20 mg</t>
+          <t xml:space="preserve">NOCAND 50 mg</t>
         </is>
       </c>
       <c r="B104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 gélule le matin</t>
+          <t xml:space="preserve">1 comprimé le matin pendant 7 jours</t>
         </is>
       </c>
       <c r="C104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antiulcéreux (inhibiteur de la pompe à protons)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OFLOCET (ofloxacine) 200 mg</t>
+          <t xml:space="preserve">NORMACOL lavement</t>
         </is>
       </c>
       <c r="B105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé (200 mg) par jour pendant 5 jours</t>
+          <t xml:space="preserve">1 lavement en l'absence de selles pendant 3 jours malgré les autres traitements (MOVICOL…)</t>
         </is>
       </c>
       <c r="C105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antibiotique (fluoroquinolone)</t>
+          <t xml:space="preserve">Laxatif (lavement rectal)</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">OLANZAPINE (ZYPREXA) 5 mg</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 comprimé le soir, de J1 à J4 de la chimiothérapie</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Antiémétique (neuroleptique)</t>
+      <c r="A106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">OEDES (oméprazole) 20 mg</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 gélule le matin</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Antiulcéreux (inhibiteur de la pompe à protons)</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OMIX (tamsulosine) 0,4 mg</t>
+          <t xml:space="preserve">OFLOCET (ofloxacine) 200 mg</t>
         </is>
       </c>
       <c r="B107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé le soir</t>
+          <t xml:space="preserve">1 comprimé (200 mg) par jour pendant 5 jours</t>
         </is>
       </c>
       <c r="C107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alpha-bloquant (troubles urinaires)</t>
+          <t xml:space="preserve">Antibiotique (fluoroquinolone)</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ORGOVYX (rélugolix) 120 mg</t>
+          <t xml:space="preserve">OLANZAPINE (ZYPREXA) 5 mg</t>
         </is>
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">3 comprimés le 1er jour, puis 1 comprimé par jour</t>
+          <t xml:space="preserve">1 comprimé le soir, de J1 à J4 de la chimiothérapie</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hormonothérapie anticancéreuse (antagoniste de la GnRH)</t>
+          <t xml:space="preserve">Antiémétique (neuroleptique)</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OROCAL VITAMINE D3 500 mg / 400 UI</t>
+          <t xml:space="preserve">OMIX (tamsulosine) 0,4 mg</t>
         </is>
       </c>
       <c r="B109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé matin et soir (soit 2 comprimés par jour)</t>
+          <t xml:space="preserve">1 comprimé le soir</t>
         </is>
       </c>
       <c r="C109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Calcium + vitamine D</t>
+          <t xml:space="preserve">Alpha-bloquant (troubles urinaires)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PARACÉTAMOL 1 g</t>
+          <t xml:space="preserve">ORGOVYX (rélugolix) 120 mg</t>
         </is>
       </c>
       <c r="B110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé en cas de douleur, maximum 4 comprimés par jour (au moins 4 heures entre 2 prises)</t>
+          <t xml:space="preserve">3 comprimés le 1er jour, puis 1 comprimé par jour</t>
         </is>
       </c>
       <c r="C110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antalgique et antipyrétique (palier 1)</t>
+          <t xml:space="preserve">Hormonothérapie anticancéreuse (antagoniste de la GnRH)</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PARACÉTAMOL CODÉINÉ</t>
+          <t xml:space="preserve">OROCAL VITAMINE D3 500 mg / 400 UI</t>
         </is>
       </c>
       <c r="B111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé en cas de douleur, maximum 4 comprimés par jour</t>
+          <t xml:space="preserve">1 comprimé matin et soir (soit 2 comprimés par jour)</t>
         </is>
       </c>
       <c r="C111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antalgique de palier 2 (paracétamol + codéine)</t>
+          <t xml:space="preserve">Calcium + vitamine D</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PENTASA (mésalazine) 1 g / 100 ml, suspension rectale</t>
+          <t xml:space="preserve">PARACÉTAMOL 1 g</t>
         </is>
       </c>
       <c r="B112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 lavement par jour, allongé sur le côté, pendant 2 semaines, puis selon les symptômes</t>
+          <t xml:space="preserve">1 comprimé en cas de douleur, maximum 4 comprimés par jour (au moins 4 heures entre 2 prises)</t>
         </is>
       </c>
       <c r="C112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Anti-inflammatoire intestinal (rectite)</t>
+          <t xml:space="preserve">Antalgique et antipyrétique (palier 1)</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PENTASA (mésalazine) 1 g, suppositoire</t>
+          <t xml:space="preserve">PARACÉTAMOL CODÉINÉ</t>
         </is>
       </c>
       <c r="B113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 suppositoire le soir pendant 7 jours</t>
+          <t xml:space="preserve">1 comprimé en cas de douleur, maximum 4 comprimés par jour</t>
         </is>
       </c>
       <c r="C113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Anti-inflammatoire intestinal (rectite)</t>
+          <t xml:space="preserve">Antalgique de palier 2 (paracétamol + codéine)</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PRIMPERAN (métoclopramide) 10 mg</t>
+          <t xml:space="preserve">PEMORIAL (pembrolizumab) 100 mg</t>
         </is>
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé matin, midi et soir (soit 3 comprimés par jour) en cas de nausées</t>
+          <t xml:space="preserve">2 flacons de 100 mg tous les 21 jours</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antiémétique (antidopaminergique)</t>
+          <t xml:space="preserve">Immunothérapie</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">PROLIA (dénosumab) 60 mg</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 injection sous-cutanée tous les 6 mois, avec calcium et vitamine D</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Anti-résorptif osseux (ostéoporose sous hormonothérapie)</t>
+      <c r="A115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PENTASA (mésalazine) 1 g / 100 ml, suspension rectale</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 lavement par jour, allongé sur le côté, pendant 2 semaines, puis selon les symptômes</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Anti-inflammatoire intestinal (rectite)</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PYOSTACINE (pristinamycine) 500 mg</t>
+          <t xml:space="preserve">PENTASA (mésalazine) 1 g, suppositoire</t>
         </is>
       </c>
       <c r="B116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2 comprimés matin et soir (soit 4 comprimés = 2 g par jour) pendant 8 à 14 jours</t>
+          <t xml:space="preserve">1 suppositoire le soir pendant 7 jours</t>
         </is>
       </c>
       <c r="C116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antibiotique (synergistine)</t>
+          <t xml:space="preserve">Anti-inflammatoire intestinal (rectite)</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RECTOLAX microlavement</t>
+          <t xml:space="preserve">PRIMPERAN (métoclopramide) 10 mg</t>
         </is>
       </c>
       <c r="B117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 lavement avant chaque séance de radiothérapie (quantité : au moins 10 lavements)</t>
+          <t xml:space="preserve">1 comprimé matin, midi et soir (soit 3 comprimés par jour) en cas de nausées</t>
         </is>
       </c>
       <c r="C117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Laxatif (lavement rectal)</t>
+          <t xml:space="preserve">Antiémétique (antidopaminergique)</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SCOPODERM (scopolamine) 1 mg / 72 h</t>
+          <t xml:space="preserve">PROLIA (dénosumab) 60 mg</t>
         </is>
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 patch derrière l'oreille, à changer toutes les 72 heures (garder 3 jours), pendant 1 mois</t>
+          <t xml:space="preserve">1 injection sous-cutanée tous les 6 mois, avec calcium et vitamine D</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Anticholinergique (antiémétique, anti-sécrétoire)</t>
+          <t xml:space="preserve">Anti-résorptif osseux (ostéoporose sous hormonothérapie)</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SEDASTERIL crème lavante PM</t>
+          <t xml:space="preserve">PYOSTACINE (pristinamycine) 500 mg</t>
         </is>
       </c>
       <c r="B119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pour la toilette intime, chaque jour</t>
+          <t xml:space="preserve">2 comprimés matin et soir (soit 4 comprimés = 2 g par jour) pendant 8 à 14 jours</t>
         </is>
       </c>
       <c r="C119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hygiène intime</t>
+          <t xml:space="preserve">Antibiotique (synergistine)</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SEDASTERIL gel lubrifiant</t>
+          <t xml:space="preserve">RECTOLAX microlavement</t>
         </is>
       </c>
       <c r="B120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 à 2 applications par jour sur la zone vulvaire, ou avant les rapports sexuels</t>
+          <t xml:space="preserve">1 lavement avant chaque séance de radiothérapie (quantité : au moins 10 lavements)</t>
         </is>
       </c>
       <c r="C120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lubrifiant intime</t>
+          <t xml:space="preserve">Laxatif (lavement rectal)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SEVREDOL (sulfate de morphine) 10 mg</t>
+          <t xml:space="preserve">SCOPODERM (scopolamine) 1 mg / 72 h</t>
         </is>
       </c>
       <c r="B121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé en cas de pic de douleur, maximum 6 comprimés par jour (au moins 1 heure entre 2 prises)</t>
+          <t xml:space="preserve">1 patch derrière l'oreille, à changer toutes les 72 heures (garder 3 jours), pendant 1 mois</t>
         </is>
       </c>
       <c r="C121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antalgique de palier 3 (morphine à libération immédiate)</t>
+          <t xml:space="preserve">Anticholinergique (antiémétique, anti-sécrétoire)</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SMECTA (diosmectite) 3 g</t>
+          <t xml:space="preserve">SEDASTERIL crème lavante PM</t>
         </is>
       </c>
       <c r="B122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 à 2 sachets en cas de diarrhée légère, maximum 6 sachets par jour</t>
+          <t xml:space="preserve">Pour la toilette intime, chaque jour</t>
         </is>
       </c>
       <c r="C122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antidiarrhéique</t>
+          <t xml:space="preserve">Hygiène intime</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SPASFON LYOC (phloroglucinol)</t>
+          <t xml:space="preserve">SEDASTERIL gel lubrifiant</t>
         </is>
       </c>
       <c r="B123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 à 2 comprimés en cas de douleurs abdominales, maximum 6 comprimés par jour</t>
+          <t xml:space="preserve">1 à 2 applications par jour sur la zone vulvaire, ou avant les rapports sexuels</t>
         </is>
       </c>
       <c r="C123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antispasmodique</t>
+          <t xml:space="preserve">Lubrifiant intime</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">SULFARLEM S 25 (anétholtrithione)</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 comprimé matin, midi et soir (soit 3 comprimés par jour), avant les repas</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Sialagogue (sécheresse buccale)</t>
+      <c r="A124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">SEVREDOL (sulfate de morphine) 10 mg</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 comprimé en cas de pic de douleur, maximum 6 comprimés par jour (au moins 1 heure entre 2 prises)</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Antalgique de palier 3 (morphine à libération immédiate)</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SYMBICORT TURBUHALER (budésonide + formotérol) 200 / 6 µg</t>
+          <t xml:space="preserve">SMECTA (diosmectite) 3 g</t>
         </is>
       </c>
       <c r="B125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 inhalation matin et soir (soit 2 inhalations par jour) pendant 1 mois</t>
+          <t xml:space="preserve">1 à 2 sachets en cas de diarrhée légère, maximum 6 sachets par jour</t>
         </is>
       </c>
       <c r="C125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antiasthmatique (corticoïde + bronchodilatateur)</t>
+          <t xml:space="preserve">Antidiarrhéique</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TADALAFIL 10 mg</t>
+          <t xml:space="preserve">SPASFON LYOC (phloroglucinol)</t>
         </is>
       </c>
       <c r="B126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé au moins 30 minutes avant l'activité sexuelle (maximum 1 par jour), pendant 3 mois</t>
+          <t xml:space="preserve">1 à 2 comprimés en cas de douleurs abdominales, maximum 6 comprimés par jour</t>
         </is>
       </c>
       <c r="C126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Traitement de la dysfonction érectile (inhibiteur de la PDE5)</t>
+          <t xml:space="preserve">Antispasmodique</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TADALAFIL 20 mg</t>
+          <t xml:space="preserve">SULFARLEM S 25 (anétholtrithione)</t>
         </is>
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé au moins 30 minutes avant l'activité sexuelle (maximum 1 par jour), pendant 3 mois</t>
+          <t xml:space="preserve">1 comprimé matin, midi et soir (soit 3 comprimés par jour), avant les repas</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Traitement de la dysfonction érectile (inhibiteur de la PDE5)</t>
+          <t xml:space="preserve">Sialagogue (sécheresse buccale)</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TADALAFIL 5 mg</t>
+          <t xml:space="preserve">SYMBICORT TURBUHALER (budésonide + formotérol) 200 / 6 µg</t>
         </is>
       </c>
       <c r="B128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé par jour, le matin, pendant 3 mois</t>
+          <t xml:space="preserve">1 inhalation matin et soir (soit 2 inhalations par jour) pendant 1 mois</t>
         </is>
       </c>
       <c r="C128" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Antiasthmatique (corticoïde + bronchodilatateur)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TADALAFIL 10 mg</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 comprimé au moins 30 minutes avant l'activité sexuelle (maximum 1 par jour), pendant 3 mois</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Traitement de la dysfonction érectile (inhibiteur de la PDE5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">TAGRISSO (osimertinib) 80 mg</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 comprimé par jour, à heure fixe, pendant ou en dehors des repas</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Thérapie ciblée (inhibiteur de l'EGFR)</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TAMOXIFÈNE 20 mg</t>
+          <t xml:space="preserve">TADALAFIL 20 mg</t>
         </is>
       </c>
       <c r="B130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé par jour, à heure fixe, pendant 3 mois</t>
+          <t xml:space="preserve">1 comprimé au moins 30 minutes avant l'activité sexuelle (maximum 1 par jour), pendant 3 mois</t>
         </is>
       </c>
       <c r="C130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hormonothérapie anticancéreuse (anti-œstrogène)</t>
+          <t xml:space="preserve">Traitement de la dysfonction érectile (inhibiteur de la PDE5)</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TANGANIL B20, comprimé</t>
+          <t xml:space="preserve">TADALAFIL 5 mg</t>
         </is>
       </c>
       <c r="B131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé matin, midi et soir (soit 3 comprimés par jour) pendant 1 mois</t>
+          <t xml:space="preserve">1 comprimé par jour, le matin, pendant 3 mois</t>
         </is>
       </c>
       <c r="C131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antivertigineux (acétylleucine)</t>
+          <t xml:space="preserve">Traitement de la dysfonction érectile (inhibiteur de la PDE5)</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TAVANIC (lévofloxacine) 500 mg</t>
+          <t xml:space="preserve">TAGRISSO (osimertinib) 80 mg</t>
         </is>
       </c>
       <c r="B132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé (500 mg) le 1er jour, puis ½ comprimé (250 mg) par jour pendant 5 jours</t>
+          <t xml:space="preserve">1 comprimé par jour, à heure fixe, pendant ou en dehors des repas</t>
         </is>
       </c>
       <c r="C132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antibiotique (fluoroquinolone)</t>
+          <t xml:space="preserve">Thérapie ciblée (inhibiteur de l'EGFR)</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TEGUMA (terbinafine) 250 mg</t>
+          <t xml:space="preserve">TAMOXIFÈNE 20 mg</t>
         </is>
       </c>
       <c r="B133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé matin et soir soit 2 comprimés par jour</t>
+          <t xml:space="preserve">1 comprimé par jour, à heure fixe, pendant 3 mois</t>
         </is>
       </c>
       <c r="C133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antifongique</t>
+          <t xml:space="preserve">Hormonothérapie anticancéreuse (anti-œstrogène)</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TEMODAL (témozolomide) 75 mg/m²/jour</t>
+          <t xml:space="preserve">TANGANIL B20, comprimé</t>
         </is>
       </c>
       <c r="B134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 prise par jour, à jeun, 1 h 30 avant la radiothérapie, tous les jours du début à la fin de la radiothérapie</t>
+          <t xml:space="preserve">1 comprimé matin, midi et soir (soit 3 comprimés par jour) pendant 1 mois</t>
         </is>
       </c>
       <c r="C134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Chimiothérapie orale (agent alkylant)</t>
+          <t xml:space="preserve">Antivertigineux (acétylleucine)</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">TEMODAL (témozolomide), phase adjuvante</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 prise par jour, à jeun, 5 jours de suite (J1 à J5) tous les 28 jours : 150 mg/m² par jour au 1er cycle, puis 200 mg/m² par jour si bonne tolérance (gélules de … mg)</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Chimiothérapie orale (agent alkylant)</t>
+      <c r="A135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TAVANIC (lévofloxacine) 500 mg</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 comprimé (500 mg) le 1er jour, puis ½ comprimé (250 mg) par jour pendant 5 jours</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Antibiotique (fluoroquinolone)</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TIORFAN (racécadotril) 100 mg</t>
+          <t xml:space="preserve">TEGUMA (terbinafine) 250 mg</t>
         </is>
       </c>
       <c r="B136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 à 2 gélules si les diarrhées importantes persistent sous LOPERIUM, maximum 6 gélules par jour</t>
+          <t xml:space="preserve">1 comprimé le matin pendant 7 jours</t>
         </is>
       </c>
       <c r="C136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antidiarrhéique (anti-sécrétoire)</t>
+          <t xml:space="preserve">Antifongique</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TITANORÉINE à la lidocaïne 2 % crème</t>
+          <t xml:space="preserve">TEMODAL (témozolomide) 75 mg/m²/jour</t>
         </is>
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 application avant et après chaque selle, maximum 4 applications par jour</t>
+          <t xml:space="preserve">1 prise par jour, à jeun, 1 h 30 avant la radiothérapie, tous les jours du début à la fin de la radiothérapie</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antihémorroïdaire</t>
+          <t xml:space="preserve">Chimiothérapie orale (agent alkylant)</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TITANORÉINE suppositoire</t>
+          <t xml:space="preserve">TEMODAL (témozolomide), phase adjuvante</t>
         </is>
       </c>
       <c r="B138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 à 2 suppositoires par jour jusqu'à cicatrisation</t>
+          <t xml:space="preserve">1 prise par jour, à jeun, 5 jours de suite (J1 à J5) tous les 28 jours : 150 mg/m² par jour au 1er cycle, puis 200 mg/m² par jour si bonne tolérance (gélules de … mg)</t>
         </is>
       </c>
       <c r="C138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antihémorroïdaire</t>
+          <t xml:space="preserve">Chimiothérapie orale (agent alkylant)</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TOLÉRIANE crème légère</t>
+          <t xml:space="preserve">TIORFAN (racécadotril) 100 mg</t>
         </is>
       </c>
       <c r="B139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 application par jour, le matin</t>
+          <t xml:space="preserve">1 à 2 gélules si les diarrhées importantes persistent sous LOPERIUM, maximum 6 gélules par jour</t>
         </is>
       </c>
       <c r="C139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Soin dermatologique apaisant</t>
+          <t xml:space="preserve">Antidiarrhéique (anti-sécrétoire)</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TRAMAL (tramadol) 50 mg</t>
+          <t xml:space="preserve">TITANORÉINE à la lidocaïne 2 % crème</t>
         </is>
       </c>
       <c r="B140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé en cas de douleur, maximum 6 comprimés par jour (au moins 4 heures entre 2 prises)</t>
+          <t xml:space="preserve">1 application avant et après chaque selle, maximum 4 applications par jour</t>
         </is>
       </c>
       <c r="C140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antalgique de palier 2 (tramadol)</t>
+          <t xml:space="preserve">Antihémorroïdaire</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TRAMAL LP (tramadol) 100 mg</t>
+          <t xml:space="preserve">TITANORÉINE suppositoire</t>
         </is>
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé le matin et 1 comprimé le soir (toutes les 12 heures)</t>
+          <t xml:space="preserve">1 à 2 suppositoires par jour jusqu'à cicatrisation</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antalgique de palier 2 (tramadol à libération prolongée)</t>
+          <t xml:space="preserve">Antihémorroïdaire</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UROREC (silodosine) 4 mg</t>
+          <t xml:space="preserve">TOLÉRIANE crème légère</t>
         </is>
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 gélule le soir pendant 3 mois</t>
+          <t xml:space="preserve">1 application par jour, le matin</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alpha-bloquant (troubles urinaires)</t>
+          <t xml:space="preserve">Soin dermatologique apaisant</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UROREC (silodosine) 8 mg</t>
+          <t xml:space="preserve">TRAMAL (tramadol) 50 mg</t>
         </is>
       </c>
       <c r="B143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 gélule le soir pendant 3 mois</t>
+          <t xml:space="preserve">1 comprimé en cas de douleur, maximum 6 comprimés par jour (au moins 4 heures entre 2 prises)</t>
         </is>
       </c>
       <c r="C143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alpha-bloquant (troubles urinaires)</t>
+          <t xml:space="preserve">Antalgique de palier 2 (tramadol)</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UVEDOSE 100 000 UI, solution buvable</t>
+          <t xml:space="preserve">TRAMAL LP (tramadol) 100 mg</t>
         </is>
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 ampoule par mois à boire sur un sucre pendant 2 mois, puis 1 ampoule tous les 3 mois</t>
+          <t xml:space="preserve">1 comprimé le matin et 1 comprimé le soir (toutes les 12 heures)</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vitamine D</t>
+          <t xml:space="preserve">Antalgique de palier 2 (tramadol à libération prolongée)</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">VASELINE stérile</t>
+          <t xml:space="preserve">UROREC (silodosine) 4 mg</t>
         </is>
       </c>
       <c r="B145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 à 2 applications par jour, en couche épaisse, sur les lésions suintantes et croûteuses</t>
+          <t xml:space="preserve">1 gélule le soir pendant 3 mois</t>
         </is>
       </c>
       <c r="C145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Émollient</t>
+          <t xml:space="preserve">Alpha-bloquant (troubles urinaires)</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">VECA (solifénacine) 10 mg</t>
+          <t xml:space="preserve">UROREC (silodosine) 8 mg</t>
         </is>
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé le soir pendant 1 mois en cas de brûlures mictionnelles</t>
+          <t xml:space="preserve">1 gélule le soir pendant 3 mois</t>
         </is>
       </c>
       <c r="C146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antispasmodique urinaire (anticholinergique)</t>
+          <t xml:space="preserve">Alpha-bloquant (troubles urinaires)</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">VECA (solifénacine) 5 mg</t>
+          <t xml:space="preserve">UVEDOSE 100 000 UI, solution buvable</t>
         </is>
       </c>
       <c r="B147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé le soir pendant 1 mois en cas de brûlures mictionnelles</t>
+          <t xml:space="preserve">1 ampoule par mois à boire sur un sucre pendant 2 mois, puis 1 ampoule tous les 3 mois</t>
         </is>
       </c>
       <c r="C147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antispasmodique urinaire (anticholinergique)</t>
+          <t xml:space="preserve">Vitamine D</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">VENTOLINE (salbutamol) 2,5 mg / 2,5 ml, solution pour nébuliseur</t>
+          <t xml:space="preserve">VASELINE stérile</t>
         </is>
       </c>
       <c r="B148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 nébulisation en cas de difficulté respiratoire, maximum 4 par jour</t>
+          <t xml:space="preserve">1 à 2 applications par jour, en couche épaisse, sur les lésions suintantes et croûteuses</t>
         </is>
       </c>
       <c r="C148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Bronchodilatateur (bêta-2 agoniste)</t>
+          <t xml:space="preserve">Émollient</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">VERZENIOS (abémaciclib) 150 mg</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 comprimé matin et soir (soit 300 mg par jour), en continu, avec l'hormonothérapie</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Thérapie ciblée (inhibiteur de CDK4/6)</t>
+      <c r="A149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">VECA (solifénacine) 10 mg</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 comprimé le soir pendant 1 mois en cas de brûlures mictionnelles</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Antispasmodique urinaire (anticholinergique)</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">VITANEVRIL FORTE</t>
+          <t xml:space="preserve">VECA (solifénacine) 5 mg</t>
         </is>
       </c>
       <c r="B150" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé matin et soir (soit 2 comprimés par jour) pendant 3 mois</t>
+          <t xml:space="preserve">1 comprimé le soir pendant 1 mois en cas de brûlures mictionnelles</t>
         </is>
       </c>
       <c r="C150" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vitamines B (neurotropes)</t>
+          <t xml:space="preserve">Antispasmodique urinaire (anticholinergique)</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">XATRAL LP (alfuzosine) 10 mg</t>
+          <t xml:space="preserve">VENTOLINE (salbutamol) 2,5 mg / 2,5 ml, solution pour nébuliseur</t>
         </is>
       </c>
       <c r="B151" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé par jour, après le repas du soir</t>
+          <t xml:space="preserve">1 nébulisation en cas de difficulté respiratoire, maximum 4 par jour</t>
         </is>
       </c>
       <c r="C151" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alpha-bloquant (troubles urinaires)</t>
+          <t xml:space="preserve">Bronchodilatateur (bêta-2 agoniste)</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">XGEVA (dénosumab) 120 mg</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 injection sous-cutanée toutes les 4 semaines, avec calcium et vitamine D</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Anti-résorptif osseux (métastases osseuses)</t>
+      <c r="A152" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">VERZENIOS (abémaciclib) 150 mg</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 comprimé matin et soir (soit 300 mg par jour), en continu, avec l'hormonothérapie</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Thérapie ciblée (inhibiteur de CDK4/6)</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">XTANDI (enzalutamide) 40 mg</t>
+          <t xml:space="preserve">VITANEVRIL FORTE</t>
         </is>
       </c>
       <c r="B153" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">4 comprimés par jour en une seule prise le matin (soit 160 mg par jour)</t>
+          <t xml:space="preserve">1 comprimé matin et soir (soit 2 comprimés par jour) pendant 3 mois</t>
         </is>
       </c>
       <c r="C153" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hormonothérapie anticancéreuse (anti-androgène)</t>
+          <t xml:space="preserve">Vitamines B (neurotropes)</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">XYLITOL chewing-gum</t>
+          <t xml:space="preserve">XATRAL LP (alfuzosine) 10 mg</t>
         </is>
       </c>
       <c r="B154" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">À mâcher selon les besoins, jusqu'à 4 fois par jour</t>
+          <t xml:space="preserve">1 comprimé par jour, après le repas du soir</t>
         </is>
       </c>
       <c r="C154" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sécheresse buccale (stimulation salivaire)</t>
+          <t xml:space="preserve">Alpha-bloquant (troubles urinaires)</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">XYLOCAÏNE VISQUEUSE (lidocaïne) 2 % gel</t>
+          <t xml:space="preserve">XGEVA (dénosumab) 120 mg</t>
         </is>
       </c>
       <c r="B155" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 application sur les zones douloureuses, après les repas ou au moins 1 heure avant</t>
+          <t xml:space="preserve">1 injection sous-cutanée toutes les 4 semaines, avec calcium et vitamine D</t>
         </is>
       </c>
       <c r="C155" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Anesthésique local</t>
+          <t xml:space="preserve">Anti-résorptif osseux (métastases osseuses)</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">YOFOLVIT (acide folique)</t>
+          <t xml:space="preserve">XTANDI (enzalutamide) 40 mg</t>
         </is>
       </c>
       <c r="B156" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé par jour, le matin, pendant 3 mois</t>
+          <t xml:space="preserve">4 comprimés par jour en une seule prise le matin (soit 160 mg par jour)</t>
         </is>
       </c>
       <c r="C156" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vitamine B9 (acide folique)</t>
+          <t xml:space="preserve">Hormonothérapie anticancéreuse (anti-androgène)</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ZETALAX, microlavement</t>
+          <t xml:space="preserve">XYLITOL chewing-gum</t>
         </is>
       </c>
       <c r="B157" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 lavement avant chaque séance de radiothérapie (quantité : au moins 10 lavements)</t>
+          <t xml:space="preserve">À mâcher selon les besoins, jusqu'à 4 fois par jour</t>
         </is>
       </c>
       <c r="C157" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Laxatif (lavement rectal)</t>
+          <t xml:space="preserve">Sécheresse buccale (stimulation salivaire)</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">ZOLADEX (goséréline) 3,6 mg</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 injection sous-cutanée tous les 28 jours</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Hormonothérapie anticancéreuse (agoniste de la LH-RH)</t>
+      <c r="A158" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">XYLOCAÏNE VISQUEUSE (lidocaïne) 2 % gel</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 application sur les zones douloureuses, après les repas ou au moins 1 heure avant</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Anesthésique local</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ZOLADEX LP (goséréline) 10,8 mg</t>
+          <t xml:space="preserve">YOFOLVIT (acide folique)</t>
         </is>
       </c>
       <c r="B159" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 injection sous-cutanée tous les 3 mois</t>
+          <t xml:space="preserve">1 comprimé par jour, le matin, pendant 3 mois</t>
         </is>
       </c>
       <c r="C159" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hormonothérapie anticancéreuse (agoniste de la LH-RH)</t>
+          <t xml:space="preserve">Vitamine B9 (acide folique)</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">ZOMETA (acide zolédronique) 4 mg</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">1 perfusion intraveineuse de 15 minutes toutes les 4 semaines (ou toutes les 12 semaines)</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Bisphosphonate (métastases osseuses)</t>
+      <c r="A160" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ZETALAX, microlavement</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 lavement avant chaque séance de radiothérapie (quantité : au moins 10 lavements)</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Laxatif (lavement rectal)</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ZOPHREN (ondansétron) 8 mg</t>
+          <t xml:space="preserve">ZOLADEX (goséréline) 3,6 mg</t>
         </is>
       </c>
       <c r="B161" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé matin et soir (soit 2 comprimés par jour) à J1, J2 et J3 après la chimiothérapie (pendant 3 jours)</t>
+          <t xml:space="preserve">1 injection sous-cutanée tous les 28 jours</t>
         </is>
       </c>
       <c r="C161" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antiémétique (sétron, anti-5HT3)</t>
+          <t xml:space="preserve">Hormonothérapie anticancéreuse (agoniste de la LH-RH)</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ZOPHREN (ondansétron) 8 mg</t>
+          <t xml:space="preserve">ZOLADEX LP (goséréline) 10,8 mg</t>
         </is>
       </c>
       <c r="B162" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1 comprimé si les nausées persistent, maximum 2 comprimés par jour (espacés de 12 heures)</t>
+          <t xml:space="preserve">1 injection sous-cutanée tous les 3 mois</t>
         </is>
       </c>
       <c r="C162" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Antiémétique (sétron, anti-5HT3)</t>
+          <t xml:space="preserve">Hormonothérapie anticancéreuse (agoniste de la LH-RH)</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">ZOMETA (acide zolédronique) 4 mg</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 perfusion intraveineuse de 15 minutes toutes les 4 semaines (ou toutes les 12 semaines)</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Bisphosphonate (métastases osseuses)</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ZOPHREN (ondansétron) 8 mg</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 comprimé matin et soir (soit 2 comprimés par jour) à J1, J2 et J3 après la chimiothérapie (pendant 3 jours)</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Antiémétique (sétron, anti-5HT3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ZOPHREN (ondansétron) 8 mg</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1 comprimé si les nausées persistent, maximum 2 comprimés par jour (espacés de 12 heures)</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Antiémétique (sétron, anti-5HT3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">ZYTIGA (abiratérone) 250 mg</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr" s="2">
+      <c r="B166" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">4 comprimés le matin en une seule prise, à jeun (au moins 2 heures après un repas et 1 heure avant le suivant), avec un grand verre d'eau (soit 1 000 mg par jour)</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr" s="2">
+      <c r="C166" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Hormonothérapie anticancéreuse (inhibiteur de la synthèse des androgènes)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C163"/>
+  <autoFilter ref="A1:C166"/>
 </worksheet>
 </file>
</xml_diff>